<commit_message>
feat(telegram): add tap-to-reveal spoiler messages with correct answer and full explanation
- In sendQuizPoll, automatically post a formatted spoiler message right below each quiz poll
- Display correct answer option explicitly (e.g. '✅ Correct Answer: Option D')
- Display the complete, untruncated explanation text without Telegram's 200-char poll truncation
- Protect answers using Telegram's native <tg-spoiler> tag so users can attempt the poll first before tapping to reveal
- Move escapeHtml helper to module scope to sanitize all HTML text sent to Telegram
</commit_message>
<xml_diff>
--- a/questions.xlsx
+++ b/questions.xlsx
@@ -571,14 +571,14 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:H7"/>
   <cols>
-    <col min="1" max="1" width="50.83203125" customWidth="1"/>
-    <col min="2" max="2" width="20.83203125" customWidth="1"/>
-    <col min="3" max="3" width="20.83203125" customWidth="1"/>
-    <col min="4" max="4" width="20.83203125" customWidth="1"/>
-    <col min="5" max="5" width="20.83203125" customWidth="1"/>
+    <col min="1" max="1" width="60.83203125" customWidth="1"/>
+    <col min="2" max="2" width="30.83203125" customWidth="1"/>
+    <col min="3" max="3" width="30.83203125" customWidth="1"/>
+    <col min="4" max="4" width="30.83203125" customWidth="1"/>
+    <col min="5" max="5" width="30.83203125" customWidth="1"/>
     <col min="6" max="6" width="15.83203125" customWidth="1"/>
-    <col min="7" max="7" width="40.83203125" customWidth="1"/>
-    <col min="8" max="8" width="25.83203125" customWidth="1"/>
+    <col min="7" max="7" width="50.83203125" customWidth="1"/>
+    <col min="8" max="8" width="30.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -662,7 +662,7 @@
         <v>Reserve Bank of India (RBI) formulates monetary policy.</v>
       </c>
       <c r="H3" t="str">
-        <v/>
+        <v>YES | 4/9/2026, 11:25:45 pm</v>
       </c>
     </row>
     <row r="4">

</xml_diff>

<commit_message>
chore(questions): record posted status for test question in Polity topic
- Tested end-to-end quiz poll delivery to newly created '⚖️ Polity' forum topic (Thread ID: 12)
- Confirmed quiz poll and spoiler explanation successfully delivered
- Marked question as posted in questions.xlsx
</commit_message>
<xml_diff>
--- a/questions.xlsx
+++ b/questions.xlsx
@@ -413,16 +413,6 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:H3"/>
-  <cols>
-    <col min="1" max="1" width="65.83203125" customWidth="1"/>
-    <col min="2" max="2" width="30.83203125" customWidth="1"/>
-    <col min="3" max="3" width="30.83203125" customWidth="1"/>
-    <col min="4" max="4" width="30.83203125" customWidth="1"/>
-    <col min="5" max="5" width="30.83203125" customWidth="1"/>
-    <col min="6" max="6" width="16.83203125" customWidth="1"/>
-    <col min="7" max="7" width="60.83203125" customWidth="1"/>
-    <col min="8" max="8" width="25.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -512,16 +502,6 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:H3"/>
-  <cols>
-    <col min="1" max="1" width="65.83203125" customWidth="1"/>
-    <col min="2" max="2" width="30.83203125" customWidth="1"/>
-    <col min="3" max="3" width="30.83203125" customWidth="1"/>
-    <col min="4" max="4" width="30.83203125" customWidth="1"/>
-    <col min="5" max="5" width="30.83203125" customWidth="1"/>
-    <col min="6" max="6" width="16.83203125" customWidth="1"/>
-    <col min="7" max="7" width="60.83203125" customWidth="1"/>
-    <col min="8" max="8" width="25.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -611,16 +591,6 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:H3"/>
-  <cols>
-    <col min="1" max="1" width="65.83203125" customWidth="1"/>
-    <col min="2" max="2" width="30.83203125" customWidth="1"/>
-    <col min="3" max="3" width="30.83203125" customWidth="1"/>
-    <col min="4" max="4" width="30.83203125" customWidth="1"/>
-    <col min="5" max="5" width="30.83203125" customWidth="1"/>
-    <col min="6" max="6" width="16.83203125" customWidth="1"/>
-    <col min="7" max="7" width="60.83203125" customWidth="1"/>
-    <col min="8" max="8" width="25.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -710,16 +680,6 @@
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:H3"/>
-  <cols>
-    <col min="1" max="1" width="65.83203125" customWidth="1"/>
-    <col min="2" max="2" width="30.83203125" customWidth="1"/>
-    <col min="3" max="3" width="30.83203125" customWidth="1"/>
-    <col min="4" max="4" width="30.83203125" customWidth="1"/>
-    <col min="5" max="5" width="30.83203125" customWidth="1"/>
-    <col min="6" max="6" width="16.83203125" customWidth="1"/>
-    <col min="7" max="7" width="60.83203125" customWidth="1"/>
-    <col min="8" max="8" width="25.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -809,16 +769,6 @@
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:H3"/>
-  <cols>
-    <col min="1" max="1" width="65.83203125" customWidth="1"/>
-    <col min="2" max="2" width="30.83203125" customWidth="1"/>
-    <col min="3" max="3" width="30.83203125" customWidth="1"/>
-    <col min="4" max="4" width="30.83203125" customWidth="1"/>
-    <col min="5" max="5" width="30.83203125" customWidth="1"/>
-    <col min="6" max="6" width="16.83203125" customWidth="1"/>
-    <col min="7" max="7" width="60.83203125" customWidth="1"/>
-    <col min="8" max="8" width="25.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -908,16 +858,6 @@
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:H3"/>
-  <cols>
-    <col min="1" max="1" width="65.83203125" customWidth="1"/>
-    <col min="2" max="2" width="30.83203125" customWidth="1"/>
-    <col min="3" max="3" width="30.83203125" customWidth="1"/>
-    <col min="4" max="4" width="30.83203125" customWidth="1"/>
-    <col min="5" max="5" width="30.83203125" customWidth="1"/>
-    <col min="6" max="6" width="16.83203125" customWidth="1"/>
-    <col min="7" max="7" width="60.83203125" customWidth="1"/>
-    <col min="8" max="8" width="25.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1007,16 +947,6 @@
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:H3"/>
-  <cols>
-    <col min="1" max="1" width="65.83203125" customWidth="1"/>
-    <col min="2" max="2" width="30.83203125" customWidth="1"/>
-    <col min="3" max="3" width="30.83203125" customWidth="1"/>
-    <col min="4" max="4" width="30.83203125" customWidth="1"/>
-    <col min="5" max="5" width="30.83203125" customWidth="1"/>
-    <col min="6" max="6" width="16.83203125" customWidth="1"/>
-    <col min="7" max="7" width="60.83203125" customWidth="1"/>
-    <col min="8" max="8" width="25.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1106,16 +1036,6 @@
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:H3"/>
-  <cols>
-    <col min="1" max="1" width="65.83203125" customWidth="1"/>
-    <col min="2" max="2" width="30.83203125" customWidth="1"/>
-    <col min="3" max="3" width="30.83203125" customWidth="1"/>
-    <col min="4" max="4" width="30.83203125" customWidth="1"/>
-    <col min="5" max="5" width="30.83203125" customWidth="1"/>
-    <col min="6" max="6" width="16.83203125" customWidth="1"/>
-    <col min="7" max="7" width="60.83203125" customWidth="1"/>
-    <col min="8" max="8" width="25.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1205,16 +1125,6 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:H3"/>
-  <cols>
-    <col min="1" max="1" width="65.83203125" customWidth="1"/>
-    <col min="2" max="2" width="30.83203125" customWidth="1"/>
-    <col min="3" max="3" width="30.83203125" customWidth="1"/>
-    <col min="4" max="4" width="30.83203125" customWidth="1"/>
-    <col min="5" max="5" width="30.83203125" customWidth="1"/>
-    <col min="6" max="6" width="16.83203125" customWidth="1"/>
-    <col min="7" max="7" width="60.83203125" customWidth="1"/>
-    <col min="8" max="8" width="25.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1304,16 +1214,6 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:H3"/>
-  <cols>
-    <col min="1" max="1" width="65.83203125" customWidth="1"/>
-    <col min="2" max="2" width="30.83203125" customWidth="1"/>
-    <col min="3" max="3" width="30.83203125" customWidth="1"/>
-    <col min="4" max="4" width="30.83203125" customWidth="1"/>
-    <col min="5" max="5" width="30.83203125" customWidth="1"/>
-    <col min="6" max="6" width="16.83203125" customWidth="1"/>
-    <col min="7" max="7" width="60.83203125" customWidth="1"/>
-    <col min="8" max="8" width="25.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1403,16 +1303,6 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:H3"/>
-  <cols>
-    <col min="1" max="1" width="65.83203125" customWidth="1"/>
-    <col min="2" max="2" width="30.83203125" customWidth="1"/>
-    <col min="3" max="3" width="30.83203125" customWidth="1"/>
-    <col min="4" max="4" width="30.83203125" customWidth="1"/>
-    <col min="5" max="5" width="30.83203125" customWidth="1"/>
-    <col min="6" max="6" width="16.83203125" customWidth="1"/>
-    <col min="7" max="7" width="60.83203125" customWidth="1"/>
-    <col min="8" max="8" width="25.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1502,16 +1392,6 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:H3"/>
-  <cols>
-    <col min="1" max="1" width="65.83203125" customWidth="1"/>
-    <col min="2" max="2" width="30.83203125" customWidth="1"/>
-    <col min="3" max="3" width="30.83203125" customWidth="1"/>
-    <col min="4" max="4" width="30.83203125" customWidth="1"/>
-    <col min="5" max="5" width="30.83203125" customWidth="1"/>
-    <col min="6" max="6" width="16.83203125" customWidth="1"/>
-    <col min="7" max="7" width="60.83203125" customWidth="1"/>
-    <col min="8" max="8" width="25.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1601,16 +1481,6 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:H3"/>
-  <cols>
-    <col min="1" max="1" width="65.83203125" customWidth="1"/>
-    <col min="2" max="2" width="30.83203125" customWidth="1"/>
-    <col min="3" max="3" width="30.83203125" customWidth="1"/>
-    <col min="4" max="4" width="30.83203125" customWidth="1"/>
-    <col min="5" max="5" width="30.83203125" customWidth="1"/>
-    <col min="6" max="6" width="16.83203125" customWidth="1"/>
-    <col min="7" max="7" width="60.83203125" customWidth="1"/>
-    <col min="8" max="8" width="25.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1701,14 +1571,14 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:H3"/>
   <cols>
-    <col min="1" max="1" width="65.83203125" customWidth="1"/>
+    <col min="1" max="1" width="60.83203125" customWidth="1"/>
     <col min="2" max="2" width="30.83203125" customWidth="1"/>
     <col min="3" max="3" width="30.83203125" customWidth="1"/>
     <col min="4" max="4" width="30.83203125" customWidth="1"/>
     <col min="5" max="5" width="30.83203125" customWidth="1"/>
-    <col min="6" max="6" width="16.83203125" customWidth="1"/>
-    <col min="7" max="7" width="60.83203125" customWidth="1"/>
-    <col min="8" max="8" width="25.83203125" customWidth="1"/>
+    <col min="6" max="6" width="15.83203125" customWidth="1"/>
+    <col min="7" max="7" width="50.83203125" customWidth="1"/>
+    <col min="8" max="8" width="30.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1760,7 +1630,7 @@
         <v>The 42nd Amendment Act (1976) introduced extensive changes across the Preamble, Fundamental Duties, and DPSP, earning the title Mini-Constitution.</v>
       </c>
       <c r="H2" t="str">
-        <v/>
+        <v>YES | 5/9/2026, 12:37:10 am</v>
       </c>
     </row>
     <row r="3">
@@ -1799,16 +1669,6 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:H3"/>
-  <cols>
-    <col min="1" max="1" width="65.83203125" customWidth="1"/>
-    <col min="2" max="2" width="30.83203125" customWidth="1"/>
-    <col min="3" max="3" width="30.83203125" customWidth="1"/>
-    <col min="4" max="4" width="30.83203125" customWidth="1"/>
-    <col min="5" max="5" width="30.83203125" customWidth="1"/>
-    <col min="6" max="6" width="16.83203125" customWidth="1"/>
-    <col min="7" max="7" width="60.83203125" customWidth="1"/>
-    <col min="8" max="8" width="25.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1898,16 +1758,6 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:H3"/>
-  <cols>
-    <col min="1" max="1" width="65.83203125" customWidth="1"/>
-    <col min="2" max="2" width="30.83203125" customWidth="1"/>
-    <col min="3" max="3" width="30.83203125" customWidth="1"/>
-    <col min="4" max="4" width="30.83203125" customWidth="1"/>
-    <col min="5" max="5" width="30.83203125" customWidth="1"/>
-    <col min="6" max="6" width="16.83203125" customWidth="1"/>
-    <col min="7" max="7" width="60.83203125" customWidth="1"/>
-    <col min="8" max="8" width="25.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">

</xml_diff>